<commit_message>
Update sitting code per RE potential data
</commit_message>
<xml_diff>
--- a/outputs_processed_data/p1_b_ember_2024_30_50.xlsx
+++ b/outputs_processed_data/p1_b_ember_2024_30_50.xlsx
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="U3">
-        <v>224948.8426581833</v>
+        <v>224948.8426581832</v>
       </c>
       <c r="W3">
         <v>60.36830343223809</v>
@@ -1994,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>204199.3492318431</v>
+        <v>204199.349231843</v>
       </c>
       <c r="AI3">
         <v>799010.6069763988</v>
@@ -2012,7 +2012,7 @@
         <v>0</v>
       </c>
       <c r="AN3">
-        <v>147895.9639373561</v>
+        <v>147895.963937356</v>
       </c>
     </row>
     <row r="4" spans="1:40">
@@ -2181,7 +2181,7 @@
         <v>0</v>
       </c>
       <c r="U5">
-        <v>642008.4255763417</v>
+        <v>642008.4255763418</v>
       </c>
       <c r="V5">
         <v>3300</v>
@@ -2238,7 +2238,7 @@
         <v>0</v>
       </c>
       <c r="AN5">
-        <v>422097.9927458331</v>
+        <v>422097.9927458332</v>
       </c>
     </row>
     <row r="6" spans="1:40">
@@ -2345,16 +2345,16 @@
         <v>109847923.4591715</v>
       </c>
       <c r="AI6">
-        <v>2190022.675978827</v>
+        <v>0</v>
       </c>
       <c r="AJ6">
-        <v>302585499.6266484</v>
+        <v>321090785.1642845</v>
       </c>
       <c r="AK6">
-        <v>44014231.1806074</v>
+        <v>2036979.139820878</v>
       </c>
       <c r="AL6">
-        <v>8561510.165999522</v>
+        <v>34223499.34512874</v>
       </c>
       <c r="AM6">
         <v>80584747.39681906</v>
@@ -2571,16 +2571,16 @@
         <v>3195311.87981393</v>
       </c>
       <c r="AI8">
-        <v>6720700.369653112</v>
+        <v>6720700.369653113</v>
       </c>
       <c r="AJ8">
-        <v>5869168.323030702</v>
+        <v>5869168.323030703</v>
       </c>
       <c r="AK8">
-        <v>3611086.126469829</v>
+        <v>3611086.126469828</v>
       </c>
       <c r="AL8">
-        <v>619181.731533197</v>
+        <v>619181.7315331971</v>
       </c>
       <c r="AM8">
         <v>5223555.028244963</v>
@@ -2639,7 +2639,7 @@
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -3130,10 +3130,10 @@
         <v>18875641.71767978</v>
       </c>
       <c r="AJ13">
-        <v>9981748.77571724</v>
+        <v>9981748.775717242</v>
       </c>
       <c r="AK13">
-        <v>6141407.527955673</v>
+        <v>6141407.527955674</v>
       </c>
       <c r="AL13">
         <v>1053048.089697059</v>
@@ -3195,13 +3195,13 @@
         <v>260000</v>
       </c>
       <c r="Q14">
-        <v>25648.25627919203</v>
+        <v>25648.25627919201</v>
       </c>
       <c r="R14">
         <v>0</v>
       </c>
       <c r="S14">
-        <v>9881.45149493586</v>
+        <v>9881.451494935862</v>
       </c>
       <c r="T14">
         <v>0</v>
@@ -3216,13 +3216,13 @@
         <v>260000</v>
       </c>
       <c r="AD14">
-        <v>25648.25627919203</v>
+        <v>25648.25627919201</v>
       </c>
       <c r="AE14">
         <v>0</v>
       </c>
       <c r="AF14">
-        <v>9881.45149493586</v>
+        <v>9881.451494935862</v>
       </c>
       <c r="AG14">
         <v>0</v>
@@ -3234,7 +3234,7 @@
         <v>286424.342787744</v>
       </c>
       <c r="AJ14">
-        <v>28254.94210930463</v>
+        <v>28254.94210930461</v>
       </c>
       <c r="AK14">
         <v>0</v>
@@ -3460,7 +3460,7 @@
         <v>710326.6435279924</v>
       </c>
       <c r="AJ16">
-        <v>206705.8106348029</v>
+        <v>206705.810634803</v>
       </c>
       <c r="AK16">
         <v>190164.6987568967</v>
@@ -3552,7 +3552,7 @@
         <v>99246.68717788679</v>
       </c>
       <c r="AF17">
-        <v>17474.44448765756</v>
+        <v>17474.44448765757</v>
       </c>
       <c r="AG17">
         <v>0</v>
@@ -3989,19 +3989,19 @@
         <v>0</v>
       </c>
       <c r="U21">
-        <v>2436083.738639096</v>
+        <v>2436083.738639095</v>
       </c>
       <c r="W21">
         <v>89.49593836999999</v>
       </c>
       <c r="AC21">
-        <v>7948580.752319796</v>
+        <v>7948580.752319794</v>
       </c>
       <c r="AD21">
-        <v>3742593.197986537</v>
+        <v>3742593.197986536</v>
       </c>
       <c r="AE21">
-        <v>5262562.920187896</v>
+        <v>5262562.920187895</v>
       </c>
       <c r="AF21">
         <v>1887476.514225975</v>
@@ -4010,16 +4010,16 @@
         <v>0</v>
       </c>
       <c r="AH21">
-        <v>2211377.076788363</v>
+        <v>2211377.076788362</v>
       </c>
       <c r="AI21">
-        <v>8205811.973943212</v>
+        <v>8205811.97394321</v>
       </c>
       <c r="AJ21">
-        <v>3863710.646541941</v>
+        <v>3863710.64654194</v>
       </c>
       <c r="AK21">
-        <v>5432869.48572602</v>
+        <v>5432869.485726019</v>
       </c>
       <c r="AL21">
         <v>1948558.851396438</v>
@@ -4028,7 +4028,7 @@
         <v>0</v>
       </c>
       <c r="AN21">
-        <v>1601639.503900958</v>
+        <v>1601639.503900957</v>
       </c>
     </row>
     <row r="22" spans="1:40">
@@ -4138,13 +4138,13 @@
         <v>6608037.433155081</v>
       </c>
       <c r="AJ22">
-        <v>4199645.423118813</v>
+        <v>6167691.368138067</v>
       </c>
       <c r="AK22">
-        <v>2583889.315971409</v>
+        <v>965030.7011529466</v>
       </c>
       <c r="AL22">
-        <v>443051.4822191052</v>
+        <v>93864.15201831431</v>
       </c>
       <c r="AM22">
         <v>0</v>
@@ -4248,7 +4248,7 @@
         <v>23857957.54465421</v>
       </c>
       <c r="AL23">
-        <v>4090849.939872771</v>
+        <v>4090849.93987277</v>
       </c>
       <c r="AM23">
         <v>31188601.65658884</v>
@@ -4411,7 +4411,7 @@
         <v>0</v>
       </c>
       <c r="Q25">
-        <v>10992.10983393944</v>
+        <v>10992.10983393943</v>
       </c>
       <c r="R25">
         <v>0</v>
@@ -4453,10 +4453,10 @@
         <v>313853.6182113793</v>
       </c>
       <c r="AK25">
-        <v>237522.54571865</v>
+        <v>237522.5457186501</v>
       </c>
       <c r="AL25">
-        <v>22907.82976934327</v>
+        <v>22907.82976934328</v>
       </c>
       <c r="AM25">
         <v>0</v>
@@ -4744,7 +4744,7 @@
         <v>90000</v>
       </c>
       <c r="R28">
-        <v>3974.804382483128</v>
+        <v>3974.804382483129</v>
       </c>
       <c r="S28">
         <v>0</v>
@@ -4845,7 +4845,7 @@
         <v>0</v>
       </c>
       <c r="Q29">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="R29">
         <v>0</v>
@@ -4884,10 +4884,10 @@
         <v>2150492.714664199</v>
       </c>
       <c r="AJ29">
-        <v>3582930.705575098</v>
+        <v>3582930.705575099</v>
       </c>
       <c r="AK29">
-        <v>1724494.05581275</v>
+        <v>1724494.055812749</v>
       </c>
       <c r="AL29">
         <v>1162402.975750703</v>
@@ -4961,7 +4961,7 @@
         <v>0</v>
       </c>
       <c r="U30">
-        <v>64200.84255763417</v>
+        <v>64200.84255763418</v>
       </c>
       <c r="W30">
         <v>39.43333333333333</v>
@@ -4982,7 +4982,7 @@
         <v>0</v>
       </c>
       <c r="AH30">
-        <v>58278.89628365688</v>
+        <v>58278.89628365689</v>
       </c>
       <c r="AI30">
         <v>11176069.09700907</v>
@@ -5000,7 +5000,7 @@
         <v>0</v>
       </c>
       <c r="AN30">
-        <v>42209.79927458331</v>
+        <v>42209.79927458332</v>
       </c>
     </row>
     <row r="31" spans="1:40">
@@ -5107,16 +5107,16 @@
         <v>2348186.154018304</v>
       </c>
       <c r="AI31">
-        <v>76892.48809864988</v>
+        <v>0</v>
       </c>
       <c r="AJ31">
-        <v>1728709.766330387</v>
+        <v>3000438.115617846</v>
       </c>
       <c r="AK31">
-        <v>1658752.188710199</v>
+        <v>794612.6440016157</v>
       </c>
       <c r="AL31">
-        <v>330696.3164802255</v>
+        <v>0</v>
       </c>
       <c r="AM31">
         <v>0</v>
@@ -5175,7 +5175,7 @@
         <v>140000</v>
       </c>
       <c r="Q32">
-        <v>73280.73222626293</v>
+        <v>73280.73222626289</v>
       </c>
       <c r="R32">
         <v>0</v>
@@ -5196,7 +5196,7 @@
         <v>504305.6797883199</v>
       </c>
       <c r="AD32">
-        <v>73280.73222626293</v>
+        <v>73280.73222626289</v>
       </c>
       <c r="AE32">
         <v>29200.62185475808</v>
@@ -5214,13 +5214,13 @@
         <v>554096.1401805037</v>
       </c>
       <c r="AJ32">
-        <v>112815.4664275033</v>
+        <v>137552.4554957462</v>
       </c>
       <c r="AK32">
-        <v>51273.97097974444</v>
+        <v>29215.65800800598</v>
       </c>
       <c r="AL32">
-        <v>6226.512454160583</v>
+        <v>3547.836357656189</v>
       </c>
       <c r="AM32">
         <v>0</v>
@@ -5699,16 +5699,16 @@
         <v>5727185509.559084</v>
       </c>
       <c r="AI36">
-        <v>3006534773.811983</v>
+        <v>3089036214.783803</v>
       </c>
       <c r="AJ36">
-        <v>5926367116.42018</v>
+        <v>5843631988.029505</v>
       </c>
       <c r="AK36">
-        <v>405174074.4394385</v>
+        <v>0</v>
       </c>
       <c r="AL36">
-        <v>1881684809.860005</v>
+        <v>2287092571.7183</v>
       </c>
       <c r="AM36">
         <v>880017848.5687089</v>
@@ -6079,7 +6079,7 @@
         <v>1050000</v>
       </c>
       <c r="Q40">
-        <v>3664.036611313147</v>
+        <v>3664.036611313144</v>
       </c>
       <c r="R40">
         <v>0</v>
@@ -6305,7 +6305,7 @@
         <v>0</v>
       </c>
       <c r="Q42">
-        <v>4763.247594707091</v>
+        <v>4763.247594707087</v>
       </c>
       <c r="R42">
         <v>0</v>
@@ -6347,7 +6347,7 @@
         <v>29833.82833904373</v>
       </c>
       <c r="AK42">
-        <v>27446.45136697479</v>
+        <v>27446.4513669748</v>
       </c>
       <c r="AL42">
         <v>82773.78845297164</v>
@@ -6445,16 +6445,16 @@
         <v>326793.2604355156</v>
       </c>
       <c r="AI43">
-        <v>10701.00291910715</v>
+        <v>7068.872372355312</v>
       </c>
       <c r="AJ43">
-        <v>240581.7357874694</v>
+        <v>338188.4126855027</v>
       </c>
       <c r="AK43">
-        <v>230845.8531175413</v>
+        <v>152492.2370090833</v>
       </c>
       <c r="AL43">
-        <v>46022.47027632617</v>
+        <v>30401.54003350272</v>
       </c>
       <c r="AM43">
         <v>0</v>
@@ -7019,16 +7019,16 @@
         <v>27940823.76723658</v>
       </c>
       <c r="AI48">
-        <v>44025859.44532017</v>
+        <v>8326189.836545795</v>
       </c>
       <c r="AJ48">
-        <v>73681858.75829211</v>
+        <v>137345347.1083471</v>
       </c>
       <c r="AK48">
-        <v>80912367.92535092</v>
+        <v>21358394.91436691</v>
       </c>
       <c r="AL48">
-        <v>21162092.7833043</v>
+        <v>52752247.05300767</v>
       </c>
       <c r="AM48">
         <v>57985358.9889133</v>
@@ -7248,13 +7248,13 @@
         <v>10934.62044007</v>
       </c>
       <c r="AJ50">
-        <v>109368.6405193204</v>
+        <v>89534.03320272124</v>
       </c>
       <c r="AK50">
-        <v>70000</v>
+        <v>89866.13643771919</v>
       </c>
       <c r="AL50">
-        <v>417.9559102143465</v>
+        <v>386.4267890943328</v>
       </c>
       <c r="AM50">
         <v>0</v>
@@ -7367,16 +7367,16 @@
         <v>3845333.785852297</v>
       </c>
       <c r="AI51">
-        <v>39506.12607391945</v>
+        <v>26593.35626928445</v>
       </c>
       <c r="AJ51">
-        <v>156355133.0027533</v>
+        <v>105249695.9254768</v>
       </c>
       <c r="AK51">
-        <v>167134960.0077859</v>
+        <v>112506083.9481773</v>
       </c>
       <c r="AL51">
-        <v>21818999.09986461</v>
+        <v>14687352.92891577</v>
       </c>
       <c r="AM51">
         <v>0</v>
@@ -7602,7 +7602,7 @@
         <v>20075795.50267576</v>
       </c>
       <c r="AL53">
-        <v>9117133.588664467</v>
+        <v>9117133.588664468</v>
       </c>
       <c r="AM53">
         <v>0</v>
@@ -7789,7 +7789,7 @@
         <v>6140000</v>
       </c>
       <c r="S55">
-        <v>642294.3471708309</v>
+        <v>642294.3471708311</v>
       </c>
       <c r="T55">
         <v>0</v>
@@ -7932,7 +7932,7 @@
         <v>26077.60118195906</v>
       </c>
       <c r="AF56">
-        <v>4591.504333123471</v>
+        <v>4591.504333123472</v>
       </c>
       <c r="AG56">
         <v>0</v>
@@ -7944,13 +7944,13 @@
         <v>494835.289192158</v>
       </c>
       <c r="AJ56">
-        <v>88639.93730041581</v>
+        <v>102014.6379289048</v>
       </c>
       <c r="AK56">
-        <v>40286.33410569208</v>
+        <v>28359.9298229144</v>
       </c>
       <c r="AL56">
-        <v>4892.216386763969</v>
+        <v>3443.920041052705</v>
       </c>
       <c r="AM56">
         <v>0</v>
@@ -8265,7 +8265,7 @@
         <v>0</v>
       </c>
       <c r="U59">
-        <v>642008.4255763417</v>
+        <v>642008.4255763418</v>
       </c>
       <c r="V59">
         <v>24092</v>
@@ -8322,7 +8322,7 @@
         <v>0</v>
       </c>
       <c r="AN59">
-        <v>422097.9927458331</v>
+        <v>422097.9927458332</v>
       </c>
     </row>
     <row r="60" spans="1:40">
@@ -8533,16 +8533,16 @@
         <v>381258.8038414349</v>
       </c>
       <c r="AI61">
-        <v>681941.2701944866</v>
+        <v>851903.928472965</v>
       </c>
       <c r="AJ61">
-        <v>11365.68783657478</v>
+        <v>3050.089242638447</v>
       </c>
       <c r="AK61">
-        <v>45176.38582275261</v>
+        <v>6462.09489185815</v>
       </c>
       <c r="AL61">
-        <v>136388.2540388973</v>
+        <v>13455.48528524949</v>
       </c>
       <c r="AM61">
         <v>0</v>
@@ -8863,16 +8863,16 @@
         <v>1506880.034230433</v>
       </c>
       <c r="AI64">
-        <v>1520000</v>
+        <v>2435363.230796492</v>
       </c>
       <c r="AJ64">
-        <v>425586.3363692678</v>
+        <v>0</v>
       </c>
       <c r="AK64">
-        <v>408363.6713849396</v>
+        <v>0</v>
       </c>
       <c r="AL64">
-        <v>81413.22304228439</v>
+        <v>0</v>
       </c>
       <c r="AM64">
         <v>0</v>
@@ -8985,16 +8985,16 @@
         <v>88733447.79881014</v>
       </c>
       <c r="AI65">
-        <v>68055676.59966424</v>
+        <v>10149698.63013699</v>
       </c>
       <c r="AJ65">
-        <v>113898259.2070554</v>
+        <v>107768330.6865833</v>
       </c>
       <c r="AK65">
-        <v>212916504.8543689</v>
+        <v>309665016.1811089</v>
       </c>
       <c r="AL65">
-        <v>32712604.83674067</v>
+        <v>0</v>
       </c>
       <c r="AM65">
         <v>87912824.92063212</v>
@@ -9053,7 +9053,7 @@
         <v>11340000</v>
       </c>
       <c r="Q66">
-        <v>238162.3797353545</v>
+        <v>238162.3797353544</v>
       </c>
       <c r="R66">
         <v>93150</v>
@@ -9110,7 +9110,7 @@
         <v>13808143.68723957</v>
       </c>
       <c r="AJ66">
-        <v>1042325.168689836</v>
+        <v>1042325.168689835</v>
       </c>
       <c r="AK66">
         <v>3510426.35669307</v>
@@ -9229,16 +9229,16 @@
         <v>14339144.67108751</v>
       </c>
       <c r="AI67">
-        <v>5639295.767496295</v>
+        <v>2854145.803588679</v>
       </c>
       <c r="AJ67">
-        <v>5302624.363597448</v>
+        <v>8546146.213181159</v>
       </c>
       <c r="AK67">
-        <v>4878295.20431832</v>
+        <v>9955732.759443711</v>
       </c>
       <c r="AL67">
-        <v>7354174.728673047</v>
+        <v>1818365.287871564</v>
       </c>
       <c r="AM67">
         <v>0</v>
@@ -9401,7 +9401,7 @@
         <v>0</v>
       </c>
       <c r="Q69">
-        <v>42136.42103010118</v>
+        <v>42136.42103010116</v>
       </c>
       <c r="R69">
         <v>0</v>
@@ -9422,13 +9422,13 @@
         <v>610711.2931188598</v>
       </c>
       <c r="AD69">
-        <v>42136.42103010118</v>
+        <v>42136.42103010116</v>
       </c>
       <c r="AE69">
         <v>35361.78601097557</v>
       </c>
       <c r="AF69">
-        <v>6226.178265534078</v>
+        <v>6226.178265534079</v>
       </c>
       <c r="AG69">
         <v>0</v>
@@ -9440,13 +9440,13 @@
         <v>671007.2558053348</v>
       </c>
       <c r="AJ69">
-        <v>100072.7536471934</v>
+        <v>100608.6631617902</v>
       </c>
       <c r="AK69">
-        <v>45482.48240117538</v>
+        <v>45004.60452505649</v>
       </c>
       <c r="AL69">
-        <v>5523.216511335427</v>
+        <v>5465.184872857544</v>
       </c>
       <c r="AM69">
         <v>0</v>
@@ -9505,7 +9505,7 @@
         <v>0</v>
       </c>
       <c r="Q70">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="R70">
         <v>0</v>
@@ -9523,16 +9523,16 @@
         <v>60</v>
       </c>
       <c r="AC70">
-        <v>84833.91875074671</v>
+        <v>84833.91875074673</v>
       </c>
       <c r="AD70">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="AE70">
-        <v>4912.106448885565</v>
+        <v>4912.106448885566</v>
       </c>
       <c r="AF70">
-        <v>864.8785556405028</v>
+        <v>864.8785556405032</v>
       </c>
       <c r="AG70">
         <v>0</v>
@@ -9541,16 +9541,16 @@
         <v>72620.72454122569</v>
       </c>
       <c r="AI70">
-        <v>93209.63221335487</v>
+        <v>93209.63221335488</v>
       </c>
       <c r="AJ70">
-        <v>23677.09880764629</v>
+        <v>30807.42288449736</v>
       </c>
       <c r="AK70">
-        <v>10761.10320323803</v>
+        <v>4402.895272466781</v>
       </c>
       <c r="AL70">
-        <v>1306.786695766915</v>
+        <v>534.6705496870766</v>
       </c>
       <c r="AM70">
         <v>0</v>
@@ -9645,16 +9645,16 @@
         <v>980379.7813065468</v>
       </c>
       <c r="AI71">
-        <v>490000</v>
+        <v>1584453.186301332</v>
       </c>
       <c r="AJ71">
-        <v>508851.9029548076</v>
+        <v>0</v>
       </c>
       <c r="AK71">
-        <v>488259.6397585933</v>
+        <v>0</v>
       </c>
       <c r="AL71">
-        <v>97341.64358793102</v>
+        <v>0</v>
       </c>
       <c r="AM71">
         <v>0</v>
@@ -10085,7 +10085,7 @@
         <v>1063983.000224448</v>
       </c>
       <c r="AK75">
-        <v>512103.780438133</v>
+        <v>512103.7804381332</v>
       </c>
       <c r="AL75">
         <v>345185.8568418902</v>
@@ -11105,16 +11105,16 @@
         <v>334006223.4634735</v>
       </c>
       <c r="AI84">
-        <v>19438662.98811545</v>
+        <v>27772505.32171381</v>
       </c>
       <c r="AJ84">
-        <v>437096196.5808172</v>
+        <v>430501142.0017376</v>
       </c>
       <c r="AK84">
-        <v>79250187.29037516</v>
+        <v>78054433.78194657</v>
       </c>
       <c r="AL84">
-        <v>35990331.95754198</v>
+        <v>35447297.71145173</v>
       </c>
       <c r="AM84">
         <v>14325794.57373152</v>
@@ -11179,7 +11179,7 @@
         <v>0</v>
       </c>
       <c r="S85">
-        <v>494072.574746793</v>
+        <v>494072.5747467931</v>
       </c>
       <c r="T85">
         <v>0</v>
@@ -11200,7 +11200,7 @@
         <v>10354833.87947028</v>
       </c>
       <c r="AF85">
-        <v>6818174.979413333</v>
+        <v>6818174.979413335</v>
       </c>
       <c r="AG85">
         <v>0</v>
@@ -11209,16 +11209,16 @@
         <v>134829452.7013531</v>
       </c>
       <c r="AI85">
-        <v>2254000</v>
+        <v>2867829.173687813</v>
       </c>
       <c r="AJ85">
-        <v>170658239.1648674</v>
+        <v>170172480.4067035</v>
       </c>
       <c r="AK85">
-        <v>30942153.05980299</v>
+        <v>30854079.83275693</v>
       </c>
       <c r="AL85">
-        <v>14051933.48027116</v>
+        <v>14011936.29179329</v>
       </c>
       <c r="AM85">
         <v>0</v>
@@ -11277,7 +11277,7 @@
         <v>14100000</v>
       </c>
       <c r="Q86">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="R86">
         <v>0</v>
@@ -11289,7 +11289,7 @@
         <v>0</v>
       </c>
       <c r="U86">
-        <v>834610.9532492443</v>
+        <v>834610.9532492444</v>
       </c>
       <c r="V86">
         <v>2716</v>
@@ -11316,7 +11316,7 @@
         <v>13025714.28571429</v>
       </c>
       <c r="AD86">
-        <v>18320.18305656573</v>
+        <v>18320.18305656572</v>
       </c>
       <c r="AE86">
         <v>0</v>
@@ -11328,13 +11328,13 @@
         <v>0</v>
       </c>
       <c r="AH86">
-        <v>757625.6516875394</v>
+        <v>757625.6516875395</v>
       </c>
       <c r="AI86">
         <v>17972636.26402408</v>
       </c>
       <c r="AJ86">
-        <v>111061.9048032909</v>
+        <v>111061.9048032908</v>
       </c>
       <c r="AK86">
         <v>0</v>
@@ -11346,7 +11346,7 @@
         <v>0</v>
       </c>
       <c r="AN86">
-        <v>548727.390569583</v>
+        <v>548727.3905695832</v>
       </c>
     </row>
     <row r="87" spans="1:40">
@@ -11396,7 +11396,7 @@
         <v>18063</v>
       </c>
       <c r="P87">
-        <v>2217291.09589254</v>
+        <v>2217291.095892541</v>
       </c>
       <c r="Q87">
         <v>6969999.999999999</v>
@@ -11685,7 +11685,7 @@
         <v>860751.0306413226</v>
       </c>
       <c r="AK89">
-        <v>729066.7870412181</v>
+        <v>729066.787041218</v>
       </c>
       <c r="AL89">
         <v>653254.6649357134</v>
@@ -11753,7 +11753,7 @@
         <v>1750000</v>
       </c>
       <c r="S90">
-        <v>64229.43471708309</v>
+        <v>64229.4347170831</v>
       </c>
       <c r="T90">
         <v>0</v>
@@ -11792,7 +11792,7 @@
         <v>2143130.501339457</v>
       </c>
       <c r="AF90">
-        <v>78658.32035769838</v>
+        <v>78658.32035769839</v>
       </c>
       <c r="AG90">
         <v>0</v>
@@ -11801,16 +11801,16 @@
         <v>15759376.03642205</v>
       </c>
       <c r="AI90">
-        <v>1203765.18441433</v>
+        <v>0</v>
       </c>
       <c r="AJ90">
-        <v>17980355.73397527</v>
+        <v>19941563.14607694</v>
       </c>
       <c r="AK90">
-        <v>6206935.713709597</v>
+        <v>5391668.424306732</v>
       </c>
       <c r="AL90">
-        <v>78658.32035769838</v>
+        <v>136483.3820732214</v>
       </c>
       <c r="AM90">
         <v>0</v>
@@ -12030,13 +12030,13 @@
         <v>80034883.13146283</v>
       </c>
       <c r="AJ92">
-        <v>42323758.24149477</v>
+        <v>42323758.24149476</v>
       </c>
       <c r="AK92">
         <v>26040271.4309963</v>
       </c>
       <c r="AL92">
-        <v>4465044.529414507</v>
+        <v>4465044.529414506</v>
       </c>
       <c r="AM92">
         <v>0</v>
@@ -12149,16 +12149,16 @@
         <v>944069.4190359339</v>
       </c>
       <c r="AI93">
-        <v>274090529.2467365</v>
+        <v>4919313.550508633</v>
       </c>
       <c r="AJ93">
-        <v>1699447585.519157</v>
+        <v>30501292.98082309</v>
       </c>
       <c r="AK93">
-        <v>1877744360.67316</v>
+        <v>33701322.34498078</v>
       </c>
       <c r="AL93">
-        <v>2985668517.376031</v>
+        <v>53586089.3669671</v>
       </c>
       <c r="AM93">
         <v>0</v>
@@ -12375,16 +12375,16 @@
         <v>8565404.976778315</v>
       </c>
       <c r="AI95">
-        <v>7059408.858091515</v>
+        <v>7354422.348246003</v>
       </c>
       <c r="AJ95">
-        <v>4371417.151473813</v>
+        <v>6407701.634452899</v>
       </c>
       <c r="AK95">
-        <v>2172410.597543724</v>
+        <v>0</v>
       </c>
       <c r="AL95">
-        <v>239851.0066838866</v>
+        <v>80963.63109403747</v>
       </c>
       <c r="AM95">
         <v>0</v>
@@ -12443,7 +12443,7 @@
         <v>0</v>
       </c>
       <c r="Q96">
-        <v>3297.632950181832</v>
+        <v>3297.63295018183</v>
       </c>
       <c r="R96">
         <v>0</v>
@@ -12464,13 +12464,13 @@
         <v>13559.81221752944</v>
       </c>
       <c r="AD96">
-        <v>3297.632950181832</v>
+        <v>3297.63295018183</v>
       </c>
       <c r="AE96">
-        <v>1781.792621683486</v>
+        <v>1781.792621683487</v>
       </c>
       <c r="AF96">
-        <v>285.230682153457</v>
+        <v>285.2306821534571</v>
       </c>
       <c r="AG96">
         <v>0</v>
@@ -12479,16 +12479,16 @@
         <v>27232.77170295963</v>
       </c>
       <c r="AI96">
-        <v>22444.62116052412</v>
+        <v>18260.91852835441</v>
       </c>
       <c r="AJ96">
-        <v>13898.44445501803</v>
+        <v>19511.75478182088</v>
       </c>
       <c r="AK96">
-        <v>6906.942754999814</v>
+        <v>5619.480855880665</v>
       </c>
       <c r="AL96">
-        <v>762.5801378283599</v>
+        <v>620.4343423143692</v>
       </c>
       <c r="AM96">
         <v>0</v>
@@ -12815,7 +12815,7 @@
         <v>106162091.1075757</v>
       </c>
       <c r="AK99">
-        <v>15442388.43695742</v>
+        <v>15442388.43695743</v>
       </c>
       <c r="AL99">
         <v>3003804.95226226</v>
@@ -13011,7 +13011,7 @@
         <v>0</v>
       </c>
       <c r="U101">
-        <v>4691553.589176392</v>
+        <v>4691553.58917639</v>
       </c>
       <c r="W101">
         <v>50.10275</v>
@@ -13020,7 +13020,7 @@
         <v>700000</v>
       </c>
       <c r="AD101">
-        <v>2152374.959876993</v>
+        <v>2152374.959876992</v>
       </c>
       <c r="AE101">
         <v>1393965.01418051</v>
@@ -13032,13 +13032,13 @@
         <v>0</v>
       </c>
       <c r="AH101">
-        <v>4258800.260874718</v>
+        <v>4258800.260874717</v>
       </c>
       <c r="AI101">
         <v>700000</v>
       </c>
       <c r="AJ101">
-        <v>4573954.934667157</v>
+        <v>4573954.934667153</v>
       </c>
       <c r="AK101">
         <v>1578958.984845793</v>
@@ -13050,7 +13050,7 @@
         <v>0</v>
       </c>
       <c r="AN101">
-        <v>3084531.719460099</v>
+        <v>3084531.719460098</v>
       </c>
     </row>
     <row r="102" spans="1:40">
@@ -13130,7 +13130,7 @@
         <v>18044.85221416123</v>
       </c>
       <c r="AF102">
-        <v>3177.171725028647</v>
+        <v>3177.171725028648</v>
       </c>
       <c r="AG102">
         <v>0</v>
@@ -13148,7 +13148,7 @@
         <v>23088.46235126211</v>
       </c>
       <c r="AL102">
-        <v>2803.773447434825</v>
+        <v>2803.773447434826</v>
       </c>
       <c r="AM102">
         <v>0</v>
@@ -13249,10 +13249,10 @@
         <v>43510274.98656373</v>
       </c>
       <c r="AK103">
-        <v>7888875.420821341</v>
+        <v>7888875.420821338</v>
       </c>
       <c r="AL103">
-        <v>3582619.232516764</v>
+        <v>3582619.232516765</v>
       </c>
       <c r="AM103">
         <v>0</v>
@@ -13311,7 +13311,7 @@
         <v>0</v>
       </c>
       <c r="Q104">
-        <v>8793.687867151551</v>
+        <v>8793.687867151546</v>
       </c>
       <c r="R104">
         <v>0</v>
@@ -13350,7 +13350,7 @@
         <v>472092.1980343095</v>
       </c>
       <c r="AJ104">
-        <v>85854.96213557952</v>
+        <v>85854.9621355795</v>
       </c>
       <c r="AK104">
         <v>72720.21661024939</v>
@@ -13537,7 +13537,7 @@
         <v>480000</v>
       </c>
       <c r="Q106">
-        <v>54960.5491696972</v>
+        <v>54960.54916969716</v>
       </c>
       <c r="R106">
         <v>0</v>
@@ -13573,16 +13573,16 @@
         <v>0</v>
       </c>
       <c r="AI106">
-        <v>480000</v>
+        <v>760657.2000073725</v>
       </c>
       <c r="AJ106">
-        <v>441528.5059734439</v>
+        <v>248825.3121461066</v>
       </c>
       <c r="AK106">
-        <v>406196.2993356019</v>
+        <v>228913.6932437462</v>
       </c>
       <c r="AL106">
-        <v>612352.9705234034</v>
+        <v>345094.182986332</v>
       </c>
       <c r="AM106">
         <v>0</v>
@@ -13695,13 +13695,13 @@
         <v>689896.8831416441</v>
       </c>
       <c r="AI107">
-        <v>286994416.577449</v>
+        <v>4617508.284062897</v>
       </c>
       <c r="AJ107">
-        <v>842033064.1828424</v>
+        <v>13547631.67760056</v>
       </c>
       <c r="AK107">
-        <v>3867205937.066116</v>
+        <v>62220218.99774873</v>
       </c>
       <c r="AL107">
         <v>0</v>
@@ -14013,7 +14013,7 @@
         <v>0</v>
       </c>
       <c r="S110">
-        <v>290020.6013763675</v>
+        <v>290020.6013763676</v>
       </c>
       <c r="T110">
         <v>0</v>
@@ -14025,16 +14025,16 @@
         <v>58.73</v>
       </c>
       <c r="AC110">
-        <v>28303.7845814145</v>
+        <v>28303.78458141446</v>
       </c>
       <c r="AD110">
-        <v>29584.30053026898</v>
+        <v>29584.30053026894</v>
       </c>
       <c r="AE110">
-        <v>26714.04011989464</v>
+        <v>26714.04011989461</v>
       </c>
       <c r="AF110">
-        <v>290020.6013763675</v>
+        <v>290020.6013763676</v>
       </c>
       <c r="AG110">
         <v>0</v>
@@ -14043,16 +14043,16 @@
         <v>263250.1264619431</v>
       </c>
       <c r="AI110">
-        <v>18244.62213867973</v>
+        <v>29750.92383840481</v>
       </c>
       <c r="AJ110">
-        <v>83787.01920478707</v>
+        <v>76019.35719900932</v>
       </c>
       <c r="AK110">
-        <v>40327.38237111169</v>
+        <v>36588.74267716421</v>
       </c>
       <c r="AL110">
-        <v>304849.0140354747</v>
+        <v>304849.0140354749</v>
       </c>
       <c r="AM110">
         <v>0</v>
@@ -14165,16 +14165,16 @@
         <v>29289756.48239255</v>
       </c>
       <c r="AI111">
-        <v>1935416.873717952</v>
+        <v>808091.6030534351</v>
       </c>
       <c r="AJ111">
-        <v>28908863.8993311</v>
+        <v>19079241.52715588</v>
       </c>
       <c r="AK111">
-        <v>16382253.52112676</v>
+        <v>27449677.35226814</v>
       </c>
       <c r="AL111">
-        <v>110476.1883016471</v>
+        <v>0</v>
       </c>
       <c r="AM111">
         <v>0</v>
@@ -14245,7 +14245,7 @@
         <v>0</v>
       </c>
       <c r="U112">
-        <v>9764156.371198732</v>
+        <v>9764156.371198734</v>
       </c>
       <c r="V112">
         <v>934.9999999999999</v>
@@ -14284,25 +14284,25 @@
         <v>0</v>
       </c>
       <c r="AH112">
-        <v>8863501.377628462</v>
+        <v>8863501.377628464</v>
       </c>
       <c r="AI112">
-        <v>403769.6854969041</v>
+        <v>403769.6854969042</v>
       </c>
       <c r="AJ112">
         <v>1912171.808597188</v>
       </c>
       <c r="AK112">
-        <v>11282632.24679525</v>
+        <v>11282632.24679526</v>
       </c>
       <c r="AL112">
-        <v>726286.1423423955</v>
+        <v>726286.1423423956</v>
       </c>
       <c r="AM112">
         <v>0</v>
       </c>
       <c r="AN112">
-        <v>6419589.900926215</v>
+        <v>6419589.900926216</v>
       </c>
     </row>
     <row r="113" spans="1:40">
@@ -14394,7 +14394,7 @@
         <v>2252003.787671233</v>
       </c>
       <c r="AJ113">
-        <v>334109.991356314</v>
+        <v>334109.9913563139</v>
       </c>
       <c r="AK113">
         <v>151851.0408486854</v>
@@ -14471,40 +14471,40 @@
         <v>0</v>
       </c>
       <c r="U114">
-        <v>946186.0533227292</v>
+        <v>946186.0533227291</v>
       </c>
       <c r="W114">
         <v>60.36830343223809</v>
       </c>
       <c r="AC114">
-        <v>806462.8688798032</v>
+        <v>806462.8688798031</v>
       </c>
       <c r="AD114">
         <v>206935.0890681745</v>
       </c>
       <c r="AE114">
-        <v>206807.2399870346</v>
+        <v>206807.2399870345</v>
       </c>
       <c r="AF114">
-        <v>88113.17259844433</v>
+        <v>88113.1725984443</v>
       </c>
       <c r="AG114">
         <v>0</v>
       </c>
       <c r="AH114">
-        <v>858908.9592887425</v>
+        <v>858908.9592887424</v>
       </c>
       <c r="AI114">
-        <v>897678.7004032622</v>
+        <v>897678.7004032618</v>
       </c>
       <c r="AJ114">
-        <v>358444.5050520056</v>
+        <v>358444.5050520058</v>
       </c>
       <c r="AK114">
-        <v>190940.7182530578</v>
+        <v>190940.7182530579</v>
       </c>
       <c r="AL114">
-        <v>98079.30571738283</v>
+        <v>98079.30571738277</v>
       </c>
       <c r="AM114">
         <v>0</v>
@@ -14846,13 +14846,13 @@
         <v>3239057.659016974</v>
       </c>
       <c r="AJ117">
-        <v>490798.1845987943</v>
+        <v>512866.7428217281</v>
       </c>
       <c r="AK117">
-        <v>223064.9100777445</v>
+        <v>216635.4461225108</v>
       </c>
       <c r="AL117">
-        <v>76911.15005667957</v>
+        <v>61272.05578897949</v>
       </c>
       <c r="AM117">
         <v>0</v>
@@ -14965,16 +14965,16 @@
         <v>1670276.664448191</v>
       </c>
       <c r="AI118">
-        <v>16543.47613183032</v>
+        <v>0</v>
       </c>
       <c r="AJ118">
-        <v>2285737.059171806</v>
+        <v>2699438.761846714</v>
       </c>
       <c r="AK118">
-        <v>332484.4034648162</v>
+        <v>0</v>
       </c>
       <c r="AL118">
-        <v>64673.82307826164</v>
+        <v>0</v>
       </c>
       <c r="AM118">
         <v>0</v>
@@ -15036,7 +15036,7 @@
         <v>207350</v>
       </c>
       <c r="R119">
-        <v>834708.920321457</v>
+        <v>834708.9203214571</v>
       </c>
       <c r="S119">
         <v>270000</v>
@@ -15313,16 +15313,16 @@
         <v>6900481.763177715</v>
       </c>
       <c r="AI121">
-        <v>2944737.683598508</v>
+        <v>2527197.084303285</v>
       </c>
       <c r="AJ121">
-        <v>5804555.040098427</v>
+        <v>4981514.874726858</v>
       </c>
       <c r="AK121">
-        <v>560000</v>
+        <v>2061904.801241131</v>
       </c>
       <c r="AL121">
-        <v>1843008.175562904</v>
+        <v>1581684.138988564</v>
       </c>
       <c r="AM121">
         <v>0</v>
@@ -15524,10 +15524,10 @@
         <v>1264478.449409576</v>
       </c>
       <c r="AJ123">
-        <v>391010.6859419438</v>
+        <v>373862.8736124572</v>
       </c>
       <c r="AK123">
-        <v>359721.0406157686</v>
+        <v>376868.8529452553</v>
       </c>
       <c r="AL123">
         <v>1020915.643423236</v>
@@ -15625,16 +15625,16 @@
         <v>2477226.6891201</v>
       </c>
       <c r="AI124">
-        <v>90000</v>
+        <v>119570.0120984971</v>
       </c>
       <c r="AJ124">
-        <v>1819578.461532794</v>
+        <v>1631686.502037989</v>
       </c>
       <c r="AK124">
-        <v>1745943.601628628</v>
+        <v>1565655.27034058</v>
       </c>
       <c r="AL124">
-        <v>348079.189749108</v>
+        <v>686689.4684334628</v>
       </c>
       <c r="AM124">
         <v>0</v>
@@ -16154,7 +16154,7 @@
         <v>54134.55664248372</v>
       </c>
       <c r="AF129">
-        <v>9531.515175085946</v>
+        <v>9531.515175085948</v>
       </c>
       <c r="AG129">
         <v>0</v>
@@ -16172,7 +16172,7 @@
         <v>69265.38705378624</v>
       </c>
       <c r="AL129">
-        <v>8411.320342304465</v>
+        <v>8411.320342304467</v>
       </c>
       <c r="AM129">
         <v>0</v>
@@ -16389,13 +16389,13 @@
         <v>1407026.537986248</v>
       </c>
       <c r="AI131">
-        <v>66718.53199423527</v>
+        <v>2805.512450108144</v>
       </c>
       <c r="AJ131">
-        <v>82419.57947961842</v>
+        <v>1822.960607247439</v>
       </c>
       <c r="AK131">
-        <v>623339.3893560028</v>
+        <v>767849.0277725009</v>
       </c>
       <c r="AL131">
         <v>1758707.562825865</v>
@@ -16707,13 +16707,13 @@
         <v>0</v>
       </c>
       <c r="S134">
-        <v>49407.2574746793</v>
+        <v>49407.25747467931</v>
       </c>
       <c r="T134">
         <v>0</v>
       </c>
       <c r="U134">
-        <v>321004.2127881708</v>
+        <v>321004.2127881709</v>
       </c>
       <c r="W134">
         <v>39.43333333333333</v>
@@ -16728,7 +16728,7 @@
         <v>0</v>
       </c>
       <c r="AF134">
-        <v>49407.2574746793</v>
+        <v>49407.25747467931</v>
       </c>
       <c r="AG134">
         <v>0</v>
@@ -16746,13 +16746,13 @@
         <v>0</v>
       </c>
       <c r="AL134">
-        <v>49728.7624093437</v>
+        <v>49728.76240934371</v>
       </c>
       <c r="AM134">
         <v>0</v>
       </c>
       <c r="AN134">
-        <v>211048.9963729165</v>
+        <v>211048.9963729166</v>
       </c>
     </row>
     <row r="135" spans="1:40">
@@ -16972,7 +16972,7 @@
         <v>7478978.329875707</v>
       </c>
       <c r="AL136">
-        <v>1454787.401369699</v>
+        <v>1454787.401369698</v>
       </c>
       <c r="AM136">
         <v>0</v>
@@ -17296,7 +17296,7 @@
         <v>39190710.09757456</v>
       </c>
       <c r="AJ139">
-        <v>3246647.736260969</v>
+        <v>3246647.73626097</v>
       </c>
       <c r="AK139">
         <v>2749950.856250295</v>
@@ -17483,7 +17483,7 @@
         <v>1000000</v>
       </c>
       <c r="Q141">
-        <v>1832.018305656573</v>
+        <v>1832.018305656572</v>
       </c>
       <c r="R141">
         <v>0</v>
@@ -17519,16 +17519,16 @@
         <v>3277010.194922809</v>
       </c>
       <c r="AI141">
-        <v>2691372.396445796</v>
+        <v>2607320.465177513</v>
       </c>
       <c r="AJ141">
-        <v>1666585.926857194</v>
+        <v>1614538.21842343</v>
       </c>
       <c r="AK141">
-        <v>828223.1605375732</v>
+        <v>802357.6369644563</v>
       </c>
       <c r="AL141">
-        <v>110000</v>
+        <v>271965.1632751643</v>
       </c>
       <c r="AM141">
         <v>0</v>
@@ -17822,7 +17822,7 @@
         <v>0</v>
       </c>
       <c r="T144">
-        <v>36078.38559683511</v>
+        <v>36078.38559683512</v>
       </c>
       <c r="U144">
         <v>9230000</v>
@@ -17843,7 +17843,7 @@
         <v>0</v>
       </c>
       <c r="AG144">
-        <v>42085.38074145372</v>
+        <v>42085.38074145373</v>
       </c>
       <c r="AH144">
         <v>8378616.093943913</v>
@@ -17861,7 +17861,7 @@
         <v>0</v>
       </c>
       <c r="AM144">
-        <v>70319.93749824951</v>
+        <v>70319.93749824952</v>
       </c>
       <c r="AN144">
         <v>6068400.846214077</v>
@@ -18039,7 +18039,7 @@
         <v>44000000</v>
       </c>
       <c r="Q146">
-        <v>3664.036611313147</v>
+        <v>3664.036611313144</v>
       </c>
       <c r="R146">
         <v>0</v>
@@ -18060,7 +18060,7 @@
         <v>44000000</v>
       </c>
       <c r="AD146">
-        <v>3664.036611313147</v>
+        <v>3664.036611313144</v>
       </c>
       <c r="AE146">
         <v>0</v>
@@ -18078,7 +18078,7 @@
         <v>44047941.79802655</v>
       </c>
       <c r="AJ146">
-        <v>3668.028895476362</v>
+        <v>3668.028895476359</v>
       </c>
       <c r="AK146">
         <v>0</v>
@@ -18155,46 +18155,46 @@
         <v>0</v>
       </c>
       <c r="U147">
-        <v>668066.3725552601</v>
+        <v>668066.3725552597</v>
       </c>
       <c r="W147">
         <v>50.10275</v>
       </c>
       <c r="AC147">
-        <v>83081.42312318229</v>
+        <v>83081.42312318223</v>
       </c>
       <c r="AD147">
         <v>340000</v>
       </c>
       <c r="AE147">
-        <v>182923.4146466215</v>
+        <v>182923.4146466213</v>
       </c>
       <c r="AF147">
-        <v>2936.076999365281</v>
+        <v>2936.076999365279</v>
       </c>
       <c r="AG147">
         <v>0</v>
       </c>
       <c r="AH147">
-        <v>606443.3002073924</v>
+        <v>606443.3002073922</v>
       </c>
       <c r="AI147">
-        <v>83081.42312318229</v>
+        <v>83081.42312318223</v>
       </c>
       <c r="AJ147">
-        <v>664651.4940585751</v>
+        <v>694834.9244805399</v>
       </c>
       <c r="AK147">
-        <v>229442.0175373537</v>
+        <v>199258.5871153885</v>
       </c>
       <c r="AL147">
-        <v>2936.076999365281</v>
+        <v>2936.076999365279</v>
       </c>
       <c r="AM147">
         <v>0</v>
       </c>
       <c r="AN147">
-        <v>439230.1777401419</v>
+        <v>439230.1777401416</v>
       </c>
     </row>
     <row r="148" spans="1:40">
@@ -18292,7 +18292,7 @@
         <v>10535040.50801177</v>
       </c>
       <c r="AL148">
-        <v>2049243.028657052</v>
+        <v>2049243.028657051</v>
       </c>
       <c r="AM148">
         <v>0</v>
@@ -18527,16 +18527,16 @@
         <v>704518777.5951618</v>
       </c>
       <c r="AI150">
-        <v>529474459.2187666</v>
+        <v>2179074550.533812</v>
       </c>
       <c r="AJ150">
-        <v>886130624.405725</v>
+        <v>94694104.34445441</v>
       </c>
       <c r="AK150">
-        <v>973087925.8494278</v>
+        <v>117570842.4058809</v>
       </c>
       <c r="AL150">
-        <v>254504688.2342791</v>
+        <v>251858200.4240514</v>
       </c>
       <c r="AM150">
         <v>430470366.1523768</v>
@@ -18640,7 +18640,7 @@
         <v>0</v>
       </c>
       <c r="AF151">
-        <v>46626.87273695782</v>
+        <v>46626.87273695783</v>
       </c>
       <c r="AG151">
         <v>0</v>
@@ -18658,7 +18658,7 @@
         <v>0</v>
       </c>
       <c r="AL151">
-        <v>50693.96501806912</v>
+        <v>50693.96501806913</v>
       </c>
       <c r="AM151">
         <v>0</v>
@@ -18851,7 +18851,7 @@
         <v>0</v>
       </c>
       <c r="U153">
-        <v>7530214.063828212</v>
+        <v>7530214.063828211</v>
       </c>
       <c r="W153">
         <v>60</v>
@@ -18872,13 +18872,13 @@
         <v>0</v>
       </c>
       <c r="AH153">
-        <v>6835620.015821653</v>
+        <v>6835620.015821652</v>
       </c>
       <c r="AI153">
         <v>16227550.45802562</v>
       </c>
       <c r="AJ153">
-        <v>158042.2305477278</v>
+        <v>158042.2305477277</v>
       </c>
       <c r="AK153">
         <v>0</v>
@@ -18985,7 +18985,7 @@
         <v>1342522.275256969</v>
       </c>
       <c r="AK154">
-        <v>1235090.311513866</v>
+        <v>1235090.311513867</v>
       </c>
       <c r="AL154">
         <v>3724820.480383723</v>
@@ -19101,16 +19101,16 @@
         <v>64490051.90614993</v>
       </c>
       <c r="AI155">
-        <v>12013375.0971857</v>
+        <v>0</v>
       </c>
       <c r="AJ155">
-        <v>55170498.04217261</v>
+        <v>104226413.2490175</v>
       </c>
       <c r="AK155">
-        <v>26554015.0642362</v>
+        <v>0</v>
       </c>
       <c r="AL155">
-        <v>10488525.04542298</v>
+        <v>0</v>
       </c>
       <c r="AM155">
         <v>0</v>
@@ -19285,7 +19285,7 @@
         <v>0</v>
       </c>
       <c r="U157">
-        <v>1667014.005252742</v>
+        <v>1667014.005252741</v>
       </c>
       <c r="W157">
         <v>62.82165000000001</v>
@@ -19306,7 +19306,7 @@
         <v>0</v>
       </c>
       <c r="AH157">
-        <v>1513247.061022809</v>
+        <v>1513247.061022808</v>
       </c>
       <c r="AI157">
         <v>2817839.26845601</v>
@@ -19404,7 +19404,7 @@
         <v>23394.03976500734</v>
       </c>
       <c r="AF158">
-        <v>4119.007503826877</v>
+        <v>4119.007503826878</v>
       </c>
       <c r="AG158">
         <v>0</v>
@@ -19416,13 +19416,13 @@
         <v>443913.3934028739</v>
       </c>
       <c r="AJ158">
-        <v>99235.97125364916</v>
+        <v>124870.0799731084</v>
       </c>
       <c r="AK158">
-        <v>45102.16968766528</v>
+        <v>22243.88279893009</v>
       </c>
       <c r="AL158">
-        <v>5477.032808339579</v>
+        <v>2701.210977615546</v>
       </c>
       <c r="AM158">
         <v>0</v>
@@ -19630,7 +19630,7 @@
         <v>34960.7312074493</v>
       </c>
       <c r="AF160">
-        <v>6155.564221881751</v>
+        <v>6155.564221881752</v>
       </c>
       <c r="AG160">
         <v>0</v>
@@ -19642,13 +19642,13 @@
         <v>663397.043949571</v>
       </c>
       <c r="AJ160">
-        <v>147822.7586248485</v>
+        <v>185826.0578064494</v>
       </c>
       <c r="AK160">
-        <v>67184.58094349066</v>
+        <v>33296.51700031044</v>
       </c>
       <c r="AL160">
-        <v>8158.635307131995</v>
+        <v>4043.400068711352</v>
       </c>
       <c r="AM160">
         <v>0</v>
@@ -19865,16 +19865,16 @@
         <v>2930111.752415232</v>
       </c>
       <c r="AI162">
-        <v>25861860.4027732</v>
+        <v>30880601.98506705</v>
       </c>
       <c r="AJ162">
-        <v>43282515.53590868</v>
+        <v>28491895.49244317</v>
       </c>
       <c r="AK162">
-        <v>47529892.44292155</v>
+        <v>41373827.06325458</v>
       </c>
       <c r="AL162">
-        <v>12431127.89364355</v>
+        <v>28359071.73448219</v>
       </c>
       <c r="AM162">
         <v>43827380.86590263</v>
@@ -20109,16 +20109,16 @@
         <v>2115078.602263198</v>
       </c>
       <c r="AI164">
-        <v>67555075.71168989</v>
+        <v>83911461.23696268</v>
       </c>
       <c r="AJ164">
-        <v>92353783.0019369</v>
+        <v>42413932.84783562</v>
       </c>
       <c r="AK164">
-        <v>101416595.556634</v>
+        <v>161524897.6110139</v>
       </c>
       <c r="AL164">
-        <v>26524837.42555141</v>
+        <v>0</v>
       </c>
       <c r="AM164">
         <v>100916187.358257</v>
@@ -20189,7 +20189,7 @@
         <v>0</v>
       </c>
       <c r="U165">
-        <v>64200.84255763417</v>
+        <v>64200.84255763418</v>
       </c>
       <c r="W165">
         <v>62.02077895833333</v>
@@ -20210,7 +20210,7 @@
         <v>0</v>
       </c>
       <c r="AH165">
-        <v>58278.89628365688</v>
+        <v>58278.89628365689</v>
       </c>
       <c r="AI165">
         <v>308761.7759046202</v>
@@ -20222,13 +20222,13 @@
         <v>0</v>
       </c>
       <c r="AL165">
-        <v>216133.2431332341</v>
+        <v>216133.2431332342</v>
       </c>
       <c r="AM165">
         <v>0</v>
       </c>
       <c r="AN165">
-        <v>42209.79927458331</v>
+        <v>42209.79927458332</v>
       </c>
     </row>
     <row r="166" spans="1:40">
@@ -20412,7 +20412,7 @@
         <v>1369686.60401564</v>
       </c>
       <c r="AF167">
-        <v>241161.8282478285</v>
+        <v>241161.8282478286</v>
       </c>
       <c r="AG167">
         <v>0</v>
@@ -20430,7 +20430,7 @@
         <v>1627465.850483279</v>
       </c>
       <c r="AL167">
-        <v>197633.1497858504</v>
+        <v>197633.1497858505</v>
       </c>
       <c r="AM167">
         <v>0</v>
@@ -20501,46 +20501,46 @@
         <v>0</v>
       </c>
       <c r="U168">
-        <v>744846.5279745499</v>
+        <v>744846.5279745497</v>
       </c>
       <c r="W168">
         <v>60</v>
       </c>
       <c r="AC168">
-        <v>892788.3993013303</v>
+        <v>892788.3993013299</v>
       </c>
       <c r="AD168">
-        <v>60626.63917271328</v>
+        <v>60626.63917271325</v>
       </c>
       <c r="AE168">
-        <v>51694.79045973795</v>
+        <v>51694.79045973792</v>
       </c>
       <c r="AF168">
-        <v>9101.943569871153</v>
+        <v>9101.943569871151</v>
       </c>
       <c r="AG168">
         <v>0</v>
       </c>
       <c r="AH168">
-        <v>676141.1816691018</v>
+        <v>676141.1816691016</v>
       </c>
       <c r="AI168">
-        <v>980934.0363932482</v>
+        <v>980934.0363932473</v>
       </c>
       <c r="AJ168">
-        <v>145532.5538148287</v>
+        <v>145532.5538148288</v>
       </c>
       <c r="AK168">
-        <v>66143.69622541797</v>
+        <v>66143.69622541804</v>
       </c>
       <c r="AL168">
-        <v>8032.234298265621</v>
+        <v>8032.234298265629</v>
       </c>
       <c r="AM168">
         <v>0</v>
       </c>
       <c r="AN168">
-        <v>489710.4334409942</v>
+        <v>489710.433440994</v>
       </c>
     </row>
     <row r="169" spans="1:40">
@@ -20632,13 +20632,13 @@
         <v>909349.2527274368</v>
       </c>
       <c r="AJ169">
-        <v>177097.5105950569</v>
+        <v>212122.0743488226</v>
       </c>
       <c r="AK169">
-        <v>80489.78483523068</v>
+        <v>49257.90019285093</v>
       </c>
       <c r="AL169">
-        <v>9774.36773733118</v>
+        <v>5981.688625945273</v>
       </c>
       <c r="AM169">
         <v>0</v>
@@ -20751,16 +20751,16 @@
         <v>155683263.6313113</v>
       </c>
       <c r="AI170">
-        <v>67423241.40389526</v>
+        <v>13229570.00836878</v>
       </c>
       <c r="AJ170">
-        <v>132902131.7893768</v>
+        <v>145323919.0676158</v>
       </c>
       <c r="AK170">
-        <v>9086257.59777707</v>
+        <v>42112215.50185191</v>
       </c>
       <c r="AL170">
-        <v>42197845.26901592</v>
+        <v>50943771.48222862</v>
       </c>
       <c r="AM170">
         <v>0</v>
@@ -21167,16 +21167,16 @@
         <v>54465.54340591926</v>
       </c>
       <c r="AI174">
-        <v>22924.61283209493</v>
+        <v>10825.89856864137</v>
       </c>
       <c r="AJ174">
-        <v>45188.12582118752</v>
+        <v>54313.64502032173</v>
       </c>
       <c r="AK174">
-        <v>5564.72613547638</v>
+        <v>16110.0826950417</v>
       </c>
       <c r="AL174">
-        <v>14347.71222798183</v>
+        <v>6775.550732735862</v>
       </c>
       <c r="AM174">
         <v>0</v>
@@ -21381,7 +21381,7 @@
         <v>19491124.95842304</v>
       </c>
       <c r="AK176">
-        <v>6728463.073520347</v>
+        <v>6728463.073520348</v>
       </c>
       <c r="AL176">
         <v>96053.31544351934</v>
@@ -21607,7 +21607,7 @@
         <v>186225593.6167516</v>
       </c>
       <c r="AK178">
-        <v>89631911.86828762</v>
+        <v>89631911.86828761</v>
       </c>
       <c r="AL178">
         <v>53843835.81094256</v>
@@ -22029,19 +22029,19 @@
         <v>0</v>
       </c>
       <c r="U182">
-        <v>4397330.383764587</v>
+        <v>4397330.383764585</v>
       </c>
       <c r="W182">
         <v>89.49593836999999</v>
       </c>
       <c r="AC182">
-        <v>14172984.41348478</v>
+        <v>14172984.41348477</v>
       </c>
       <c r="AD182">
-        <v>6673356.755619111</v>
+        <v>6673356.755619106</v>
       </c>
       <c r="AE182">
-        <v>9383589.922142765</v>
+        <v>9383589.922142759</v>
       </c>
       <c r="AF182">
         <v>3780000</v>
@@ -22050,25 +22050,25 @@
         <v>0</v>
       </c>
       <c r="AH182">
-        <v>3991716.481451629</v>
+        <v>3991716.481451627</v>
       </c>
       <c r="AI182">
-        <v>14631649.20010927</v>
+        <v>14631649.20010926</v>
       </c>
       <c r="AJ182">
-        <v>6889319.298375663</v>
+        <v>6889319.298375659</v>
       </c>
       <c r="AK182">
-        <v>9687260.775355332</v>
+        <v>9687260.775355328</v>
       </c>
       <c r="AL182">
-        <v>3902328.003958786</v>
+        <v>3902328.003958787</v>
       </c>
       <c r="AM182">
         <v>0</v>
       </c>
       <c r="AN182">
-        <v>2891090.29489923</v>
+        <v>2891090.294899228</v>
       </c>
     </row>
     <row r="183" spans="1:40">
@@ -22246,7 +22246,7 @@
         <v>1409361.70212766</v>
       </c>
       <c r="R184">
-        <v>3974804.382483128</v>
+        <v>3974804.382483129</v>
       </c>
       <c r="S184">
         <v>0</v>
@@ -22285,7 +22285,7 @@
         <v>4787234.042553192</v>
       </c>
       <c r="AE184">
-        <v>11924413.14744938</v>
+        <v>11924413.14744939</v>
       </c>
       <c r="AF184">
         <v>0</v>
@@ -22303,7 +22303,7 @@
         <v>38862218.90627506</v>
       </c>
       <c r="AK184">
-        <v>51597061.97087711</v>
+        <v>51597061.97087712</v>
       </c>
       <c r="AL184">
         <v>0</v>
@@ -22365,7 +22365,7 @@
         <v>64980000.00000001</v>
       </c>
       <c r="Q185">
-        <v>2015.220136222231</v>
+        <v>2015.220136222229</v>
       </c>
       <c r="R185">
         <v>20000</v>
@@ -22386,7 +22386,7 @@
         <v>64980000.00000001</v>
       </c>
       <c r="AD185">
-        <v>2015.220136222231</v>
+        <v>2015.220136222229</v>
       </c>
       <c r="AE185">
         <v>20000</v>
@@ -22404,7 +22404,7 @@
         <v>69445887.83033092</v>
       </c>
       <c r="AJ185">
-        <v>2153.720399099927</v>
+        <v>2153.720399099925</v>
       </c>
       <c r="AK185">
         <v>21374.54226849213</v>
@@ -22731,16 +22731,16 @@
         <v>54465.54340591926</v>
       </c>
       <c r="AI188">
-        <v>44889.24232104824</v>
+        <v>14039.2856360056</v>
       </c>
       <c r="AJ188">
-        <v>27796.88891003608</v>
+        <v>42736.76270732118</v>
       </c>
       <c r="AK188">
-        <v>13813.88550999963</v>
+        <v>30785.15347106913</v>
       </c>
       <c r="AL188">
-        <v>1525.16027565672</v>
+        <v>463.9752023447321</v>
       </c>
       <c r="AM188">
         <v>0</v>
@@ -22835,16 +22835,16 @@
         <v>81698.3151088789</v>
       </c>
       <c r="AI189">
-        <v>35381.87145743773</v>
+        <v>33605.11390739959</v>
       </c>
       <c r="AJ189">
-        <v>69743.40072471673</v>
+        <v>98432.65161771141</v>
       </c>
       <c r="AK189">
-        <v>4768.219261780282</v>
+        <v>0</v>
       </c>
       <c r="AL189">
-        <v>22144.27408117626</v>
+        <v>0</v>
       </c>
       <c r="AM189">
         <v>0</v>
@@ -23052,7 +23052,7 @@
         <v>162955.9223460197</v>
       </c>
       <c r="AF191">
-        <v>28691.78105528771</v>
+        <v>28691.78105528772</v>
       </c>
       <c r="AG191">
         <v>0</v>
@@ -23064,13 +23064,13 @@
         <v>3132625.307688822</v>
       </c>
       <c r="AJ191">
-        <v>683309.150969674</v>
+        <v>868831.9446350051</v>
       </c>
       <c r="AK191">
-        <v>310560.0205936962</v>
+        <v>145126.7968989491</v>
       </c>
       <c r="AL191">
-        <v>37713.20611689932</v>
+        <v>17623.6361463152</v>
       </c>
       <c r="AM191">
         <v>0</v>

</xml_diff>